<commit_message>
Change of ELC_SELLING and ELC_PRICE
</commit_message>
<xml_diff>
--- a/SubRES_TMPL/SubRes_ELC_DKprices.xlsx
+++ b/SubRES_TMPL/SubRes_ELC_DKprices.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\VEDA_models\KModel_03\SubRES_TMPL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56902A1A-099B-48D9-A1F7-878138B89D60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD74DA0-623B-4100-90D9-9808816231A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Intro" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
   <si>
     <t>Description</t>
   </si>
@@ -158,6 +158,9 @@
   </si>
   <si>
     <t>Sale of electricity to Denmark West</t>
+  </si>
+  <si>
+    <t>GW</t>
   </si>
 </sst>
 </file>
@@ -384,7 +387,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="da-DK" sz="1100" kern="1200" baseline="0"/>
-            <a:t> have been using GW most places, so I might change it here too, but it was MW originally.</a:t>
+            <a:t> have been using GW most places, so I might change it here too, but it was MW originally. MW doesn't make sense for CAP2ACT. Also CAP2ACT should be 0.0036 not 0.036, right? </a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -922,7 +925,7 @@
         <v>22</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="G3" s="9" t="s">
         <v>24</v>

</xml_diff>